<commit_message>
Successfully excluded LNG from Fuel cost calculation in existing model
</commit_message>
<xml_diff>
--- a/Input/urbs_intertemporal_2050/2024.xlsx
+++ b/Input/urbs_intertemporal_2050/2024.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxoi\GitHub\urbs-extension\Input\urbs_intertemporal_2050\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCCCEC15-800B-430A-82CF-712A361B8B74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE1CACB3-5E98-40DC-AEBB-980362CE09E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="67080" yWindow="-1935" windowWidth="29040" windowHeight="17520" tabRatio="796" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-5445" windowWidth="38640" windowHeight="21120" tabRatio="796" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Global" sheetId="11" r:id="rId1"/>
@@ -365,10 +365,10 @@
     <t>Piped Gas</t>
   </si>
   <si>
-    <t xml:space="preserve">LNG </t>
-  </si>
-  <si>
     <t>Gas Plant (CCGT) LNG</t>
+  </si>
+  <si>
+    <t>LNG</t>
   </si>
 </sst>
 </file>
@@ -3390,7 +3390,7 @@
         <v>94</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>5</v>
@@ -3969,7 +3969,7 @@
         <v>94</v>
       </c>
       <c r="B12" s="59" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C12" s="50">
         <v>56670</v>
@@ -4597,10 +4597,10 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="59" t="s">
+        <v>103</v>
+      </c>
+      <c r="B29" s="4" t="s">
         <v>104</v>
-      </c>
-      <c r="B29" s="4" t="s">
-        <v>103</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>39</v>
@@ -4615,7 +4615,7 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="59" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B30" s="4" t="s">
         <v>35</v>
@@ -4633,7 +4633,7 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="59" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B31" s="4" t="s">
         <v>25</v>

</xml_diff>

<commit_message>
Model runs through, need to validate
atm seems like fossil exit to early
</commit_message>
<xml_diff>
--- a/Input/urbs_intertemporal_2050/2024.xlsx
+++ b/Input/urbs_intertemporal_2050/2024.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxoi\GitHub\urbs-extension\Input\urbs_intertemporal_2050\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{867B10B5-66B7-4BCD-B9C8-6C440BFBFF37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D83EA04-9730-41E6-B4A7-C16CB7838C92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-5445" windowWidth="38640" windowHeight="21120" tabRatio="796" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="67080" yWindow="-5565" windowWidth="38640" windowHeight="21120" tabRatio="796" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Global" sheetId="11" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="105">
   <si>
     <t>t</t>
   </si>
@@ -342,12 +342,6 @@
   </si>
   <si>
     <t>EU27.Hydro</t>
-  </si>
-  <si>
-    <t>EU27.Lignite plant</t>
-  </si>
-  <si>
-    <t>EU27.Gas plant</t>
   </si>
   <si>
     <t>Gas Plant (CCGT) CCUS</t>
@@ -1749,11 +1743,8 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -2877,80 +2868,80 @@
   <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="14.109375" style="32" customWidth="1"/>
-    <col min="2" max="2" width="17.33203125" style="32" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="74.88671875" style="32" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="11.44140625" style="32"/>
+    <col min="1" max="1" width="14.109375" style="31" customWidth="1"/>
+    <col min="2" max="2" width="17.33203125" style="31" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="74.88671875" style="31" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="11.44140625" style="31"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="B1" s="31" t="s">
+      <c r="B1" s="30" t="s">
         <v>61</v>
       </c>
-      <c r="C1" s="31" t="s">
+      <c r="C1" s="30" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" s="33" t="s">
+      <c r="A2" s="32" t="s">
         <v>65</v>
       </c>
-      <c r="B2" s="37">
+      <c r="B2" s="36">
         <v>2024</v>
       </c>
-      <c r="C2" s="29" t="s">
+      <c r="C2" s="28" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" s="33" t="s">
+      <c r="A3" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="B3" s="37">
+      <c r="B3" s="36">
         <v>0.03</v>
       </c>
-      <c r="C3" s="29" t="s">
+      <c r="C3" s="28" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="43.2">
-      <c r="A4" s="33" t="s">
+      <c r="A4" s="32" t="s">
         <v>60</v>
       </c>
-      <c r="B4" s="59" t="s">
+      <c r="B4" s="58" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="29" t="s">
+      <c r="C4" s="28" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:3">
-      <c r="A5" s="33" t="s">
+      <c r="A5" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="B5" s="38" t="s">
+      <c r="B5" s="37" t="s">
         <v>27</v>
       </c>
-      <c r="C5" s="29" t="s">
+      <c r="C5" s="28" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="28.8">
-      <c r="A6" s="33" t="s">
+      <c r="A6" s="32" t="s">
         <v>71</v>
       </c>
-      <c r="B6" s="58" t="s">
+      <c r="B6" s="57" t="s">
         <v>27</v>
       </c>
-      <c r="C6" s="29" t="s">
+      <c r="C6" s="28" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="7" spans="1:3">
-      <c r="B7" s="58"/>
+      <c r="B7" s="57"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -2969,118 +2960,118 @@
   <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="16384" width="11.44140625" style="2"/>
+    <col min="1" max="16384" width="11.44140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="15" customFormat="1">
-      <c r="A1" s="13" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="14" t="s">
+    <row r="1" spans="1:2" s="14" customFormat="1">
+      <c r="A1" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="13" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="5">
-        <v>0</v>
-      </c>
-      <c r="B2" s="27">
+      <c r="A2" s="4">
+        <v>0</v>
+      </c>
+      <c r="B2" s="26">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3" s="5">
+      <c r="A3" s="4">
         <v>1</v>
       </c>
-      <c r="B3" s="27">
+      <c r="B3" s="26">
         <v>0.33750000000000002</v>
       </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4" s="5">
+      <c r="A4" s="4">
         <v>2</v>
       </c>
-      <c r="B4" s="27">
+      <c r="B4" s="26">
         <v>0.33750000000000002</v>
       </c>
     </row>
     <row r="5" spans="1:2">
-      <c r="A5" s="5">
+      <c r="A5" s="4">
         <v>3</v>
       </c>
-      <c r="B5" s="27">
+      <c r="B5" s="26">
         <v>0.33750000000000002</v>
       </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6" s="5">
+      <c r="A6" s="4">
         <v>4</v>
       </c>
-      <c r="B6" s="27">
+      <c r="B6" s="26">
         <v>0.33750000000000002</v>
       </c>
     </row>
     <row r="7" spans="1:2">
-      <c r="A7" s="5">
+      <c r="A7" s="4">
         <v>5</v>
       </c>
-      <c r="B7" s="27">
+      <c r="B7" s="26">
         <v>0.33750000000000002</v>
       </c>
     </row>
     <row r="8" spans="1:2">
-      <c r="A8" s="5">
+      <c r="A8" s="4">
         <v>6</v>
       </c>
-      <c r="B8" s="27">
+      <c r="B8" s="26">
         <v>0.33750000000000002</v>
       </c>
     </row>
     <row r="9" spans="1:2">
-      <c r="A9" s="5">
+      <c r="A9" s="4">
         <v>7</v>
       </c>
-      <c r="B9" s="27">
+      <c r="B9" s="26">
         <v>0.33750000000000002</v>
       </c>
     </row>
     <row r="10" spans="1:2">
-      <c r="A10" s="5">
+      <c r="A10" s="4">
         <v>8</v>
       </c>
-      <c r="B10" s="27">
+      <c r="B10" s="26">
         <v>0.33750000000000002</v>
       </c>
     </row>
     <row r="11" spans="1:2">
-      <c r="A11" s="5">
+      <c r="A11" s="4">
         <v>9</v>
       </c>
-      <c r="B11" s="27">
+      <c r="B11" s="26">
         <v>0.33750000000000002</v>
       </c>
     </row>
     <row r="12" spans="1:2">
-      <c r="A12" s="5">
+      <c r="A12" s="4">
         <v>10</v>
       </c>
-      <c r="B12" s="27">
+      <c r="B12" s="26">
         <v>0.33750000000000002</v>
       </c>
     </row>
     <row r="13" spans="1:2">
-      <c r="A13" s="5">
+      <c r="A13" s="4">
         <v>11</v>
       </c>
-      <c r="B13" s="27">
+      <c r="B13" s="26">
         <v>0.33750000000000002</v>
       </c>
     </row>
     <row r="14" spans="1:2">
-      <c r="A14" s="5">
+      <c r="A14" s="4">
         <v>12</v>
       </c>
-      <c r="B14" s="27">
+      <c r="B14" s="26">
         <v>0.33750000000000002</v>
       </c>
     </row>
@@ -3099,17 +3090,17 @@
   <dimension ref="A1:C1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="16384" width="11.44140625" style="2"/>
+    <col min="1" max="16384" width="11.44140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="15" customFormat="1">
-      <c r="A1" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="15" t="s">
+    <row r="1" spans="1:3" s="14" customFormat="1">
+      <c r="A1" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C1" s="14" t="s">
         <v>80</v>
       </c>
     </row>
@@ -3124,23 +3115,86 @@
   <sheetPr>
     <tabColor theme="9" tint="0.39997558519241921"/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="11.44140625" style="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>97</v>
+    <row r="1" spans="1:2">
+      <c r="A1" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5"/>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" s="4">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" s="4">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" s="4">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" s="4">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" s="4">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Demand" prompt="Demand (MWh) of commodity Co in site Sit for each time step. Column title: &quot;Co.Sit&quot;" sqref="B1:C1" xr:uid="{2A4A1C90-4C72-401E-8036-416065416BAB}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Demand" prompt="Demand (MWh) of commodity Co in site Sit for each time step. Column title: &quot;Co.Sit&quot;" sqref="B1" xr:uid="{2A4A1C90-4C72-401E-8036-416065416BAB}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3161,15 +3215,15 @@
       <c r="A1" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="11" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="B2" s="7">
+      <c r="B2" s="6">
         <v>280000000</v>
       </c>
     </row>
@@ -3190,13 +3244,13 @@
   <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="10.6640625" style="3" customWidth="1"/>
-    <col min="2" max="2" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.6640625" style="3" customWidth="1"/>
-    <col min="4" max="4" width="10.6640625" style="9" customWidth="1"/>
-    <col min="5" max="5" width="16.33203125" style="9" customWidth="1"/>
-    <col min="6" max="6" width="13.88671875" style="10" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="11.44140625" style="3"/>
+    <col min="1" max="1" width="10.6640625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.6640625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="10.6640625" style="8" customWidth="1"/>
+    <col min="5" max="5" width="16.33203125" style="8" customWidth="1"/>
+    <col min="6" max="6" width="13.88671875" style="9" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="11.44140625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" customFormat="1">
@@ -3209,219 +3263,219 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="F1" s="10" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="28" t="e">
+      <c r="D2" s="27" t="e">
         <f>NA()</f>
         <v>#N/A</v>
       </c>
-      <c r="E2" s="28" t="e">
+      <c r="E2" s="27" t="e">
         <f>NA()</f>
         <v>#N/A</v>
       </c>
-      <c r="F2" s="28" t="e">
+      <c r="F2" s="27" t="e">
         <f>NA()</f>
         <v>#N/A</v>
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="28" t="e">
+      <c r="D3" s="27" t="e">
         <f>NA()</f>
         <v>#N/A</v>
       </c>
-      <c r="E3" s="28" t="e">
+      <c r="E3" s="27" t="e">
         <f>NA()</f>
         <v>#N/A</v>
       </c>
-      <c r="F3" s="28" t="e">
+      <c r="F3" s="27" t="e">
         <f>NA()</f>
         <v>#N/A</v>
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D4">
         <v>8.64</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4">
+        <v>372611941.46341461</v>
+      </c>
+      <c r="F4" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="F4" s="8" t="s">
-        <v>27</v>
-      </c>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="C5" s="4" t="s">
+      <c r="B5" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D5">
         <v>22.68</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="7" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="3" t="s">
         <v>26</v>
       </c>
       <c r="D6">
         <v>65</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="6" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:6">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D7">
         <v>67.680000000000007</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="7" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:6">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D8">
         <v>6.12</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="7" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D9">
         <v>6.48</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9">
+        <v>240351818.66666669</v>
+      </c>
+      <c r="F9" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="F9" s="8" t="s">
-        <v>27</v>
-      </c>
     </row>
     <row r="10" spans="1:6">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="C10" s="4" t="s">
+      <c r="B10" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C10" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D10">
         <v>33.119999999999997</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10">
+        <v>27775463.399999999</v>
+      </c>
+      <c r="F10" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="F10" s="8" t="s">
-        <v>27</v>
-      </c>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="C11" s="4" t="s">
+      <c r="B11" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="C11" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D11">
-        <v>33.119999999999997</v>
-      </c>
-      <c r="E11" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="F11" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="E11">
+        <v>184548562.5</v>
+      </c>
+      <c r="F11" s="7" t="s">
         <v>27</v>
       </c>
     </row>
@@ -3454,20 +3508,20 @@
   <dimension ref="A1:O13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="10.6640625" style="3" customWidth="1"/>
-    <col min="2" max="2" width="16.33203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="10.6640625" style="20" customWidth="1"/>
-    <col min="6" max="6" width="20.109375" style="20" customWidth="1"/>
-    <col min="7" max="7" width="18.109375" style="20" customWidth="1"/>
-    <col min="8" max="8" width="10.6640625" style="3" customWidth="1"/>
-    <col min="9" max="9" width="24" style="20" customWidth="1"/>
-    <col min="10" max="10" width="10.6640625" style="20" customWidth="1"/>
-    <col min="11" max="11" width="10.6640625" style="22" customWidth="1"/>
-    <col min="12" max="12" width="16.109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.5546875" style="3" customWidth="1"/>
-    <col min="14" max="14" width="14.88671875" style="23" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.88671875" style="3" bestFit="1" customWidth="1"/>
-    <col min="16" max="16384" width="11.44140625" style="3"/>
+    <col min="1" max="1" width="10.6640625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="16.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="10.6640625" style="19" customWidth="1"/>
+    <col min="6" max="6" width="20.109375" style="19" customWidth="1"/>
+    <col min="7" max="7" width="18.109375" style="19" customWidth="1"/>
+    <col min="8" max="8" width="10.6640625" style="2" customWidth="1"/>
+    <col min="9" max="9" width="24" style="19" customWidth="1"/>
+    <col min="10" max="10" width="10.6640625" style="19" customWidth="1"/>
+    <col min="11" max="11" width="10.6640625" style="21" customWidth="1"/>
+    <col min="12" max="12" width="16.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.5546875" style="2" customWidth="1"/>
+    <col min="14" max="14" width="14.88671875" style="22" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="16" max="16384" width="11.44140625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" customFormat="1">
@@ -3477,607 +3531,607 @@
       <c r="B1" t="s">
         <v>42</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="C1" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="16" t="s">
         <v>73</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="E1" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="17" t="s">
+      <c r="F1" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="G1" s="17" t="s">
+      <c r="G1" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="H1" s="36" t="s">
+      <c r="H1" s="35" t="s">
         <v>55</v>
       </c>
-      <c r="I1" s="17" t="s">
+      <c r="I1" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="J1" s="17" t="s">
+      <c r="J1" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="K1" s="19" t="s">
+      <c r="K1" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="L1" s="36" t="s">
+      <c r="L1" s="35" t="s">
         <v>74</v>
       </c>
-      <c r="M1" s="16" t="s">
+      <c r="M1" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="N1" s="16" t="s">
+      <c r="N1" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="O1" s="16" t="s">
+      <c r="O1" s="15" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:15">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="C2" s="20">
+      <c r="C2" s="19">
         <v>56122</v>
       </c>
-      <c r="D2" s="20">
+      <c r="D2" s="19">
         <v>5</v>
       </c>
-      <c r="E2" s="20">
-        <v>0</v>
-      </c>
-      <c r="F2" s="20">
+      <c r="E2" s="19">
+        <v>0</v>
+      </c>
+      <c r="F2" s="19">
         <v>56122</v>
       </c>
-      <c r="G2" s="50" t="s">
+      <c r="G2" s="49" t="s">
         <v>27</v>
       </c>
-      <c r="H2" s="51">
-        <v>0.5</v>
-      </c>
-      <c r="I2" s="54">
+      <c r="H2" s="50">
+        <v>0</v>
+      </c>
+      <c r="I2" s="53">
         <v>1784013.3447999998</v>
       </c>
-      <c r="J2" s="55">
+      <c r="J2" s="54">
         <v>28544.213516800002</v>
       </c>
-      <c r="K2" s="52">
+      <c r="K2" s="51">
         <v>2.7</v>
       </c>
-      <c r="L2" s="53">
-        <v>0</v>
-      </c>
-      <c r="M2" s="42">
+      <c r="L2" s="52">
+        <v>0</v>
+      </c>
+      <c r="M2" s="41">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="N2" s="53">
+      <c r="N2" s="52">
         <v>40</v>
       </c>
-      <c r="O2" s="28" t="e">
+      <c r="O2" s="27" t="e">
         <v>#N/A</v>
       </c>
     </row>
     <row r="3" spans="1:15">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="C3" s="20">
+      <c r="B3" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C3" s="19">
         <v>43599</v>
       </c>
-      <c r="D3" s="20">
+      <c r="D3" s="19">
         <v>5</v>
       </c>
-      <c r="E3" s="20">
-        <v>0</v>
-      </c>
-      <c r="F3" s="20">
+      <c r="E3" s="19">
+        <v>0</v>
+      </c>
+      <c r="F3" s="19">
         <v>43599</v>
       </c>
-      <c r="G3" s="50" t="s">
+      <c r="G3" s="49" t="s">
         <v>27</v>
       </c>
-      <c r="H3" s="51">
-        <v>0.65</v>
-      </c>
-      <c r="I3" s="52">
+      <c r="H3" s="50">
+        <v>0</v>
+      </c>
+      <c r="I3" s="51">
         <v>2230016.6809999999</v>
       </c>
-      <c r="J3" s="52">
+      <c r="J3" s="51">
         <v>52182.390330800001</v>
       </c>
-      <c r="K3" s="53">
+      <c r="K3" s="52">
         <v>4.5999999999999996</v>
       </c>
-      <c r="L3" s="53">
-        <v>0</v>
-      </c>
-      <c r="M3" s="42">
+      <c r="L3" s="52">
+        <v>0</v>
+      </c>
+      <c r="M3" s="41">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="N3" s="53">
+      <c r="N3" s="52">
         <v>40</v>
       </c>
-      <c r="O3" s="28" t="e">
+      <c r="O3" s="27" t="e">
         <v>#N/A</v>
       </c>
     </row>
     <row r="4" spans="1:15">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="C4" s="20">
+      <c r="C4" s="19">
         <v>187303</v>
       </c>
-      <c r="D4" s="20">
+      <c r="D4" s="19">
         <v>25</v>
       </c>
-      <c r="E4" s="20">
-        <v>0</v>
-      </c>
-      <c r="F4" s="20">
+      <c r="E4" s="19">
+        <v>0</v>
+      </c>
+      <c r="F4" s="19">
         <v>999999</v>
       </c>
-      <c r="G4" s="50" t="s">
+      <c r="G4" s="49" t="s">
         <v>27</v>
       </c>
-      <c r="H4" s="3">
-        <v>0.5</v>
-      </c>
-      <c r="I4" s="52">
+      <c r="H4" s="2">
+        <v>0</v>
+      </c>
+      <c r="I4" s="51">
         <v>802808.92800000007</v>
       </c>
-      <c r="J4" s="52">
+      <c r="J4" s="51">
         <v>16725.186000000002</v>
       </c>
-      <c r="K4" s="53">
+      <c r="K4" s="52">
         <v>2.6</v>
       </c>
-      <c r="L4" s="54">
-        <v>0</v>
-      </c>
-      <c r="M4" s="42">
+      <c r="L4" s="53">
+        <v>0</v>
+      </c>
+      <c r="M4" s="41">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="N4" s="53">
+      <c r="N4" s="52">
         <v>25</v>
       </c>
-      <c r="O4" s="28" t="e">
+      <c r="O4" s="27" t="e">
         <v>#N/A</v>
       </c>
     </row>
     <row r="5" spans="1:15">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="C5" s="20">
+      <c r="B5" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C5" s="19">
         <v>13483</v>
       </c>
-      <c r="D5" s="20">
+      <c r="D5" s="19">
         <v>10</v>
       </c>
-      <c r="E5" s="20">
-        <v>0</v>
-      </c>
-      <c r="F5" s="20">
+      <c r="E5" s="19">
+        <v>0</v>
+      </c>
+      <c r="F5" s="19">
         <v>13483</v>
       </c>
-      <c r="G5" s="50" t="s">
+      <c r="G5" s="49" t="s">
         <v>27</v>
       </c>
-      <c r="H5" s="3">
+      <c r="H5" s="2">
         <v>0</v>
       </c>
       <c r="I5">
         <v>5648000</v>
       </c>
-      <c r="J5" s="60">
+      <c r="J5" s="59">
         <v>16725.186000000002</v>
       </c>
       <c r="K5">
         <v>2.6</v>
       </c>
-      <c r="L5" s="54">
-        <v>0</v>
-      </c>
-      <c r="M5" s="42">
+      <c r="L5" s="53">
+        <v>0</v>
+      </c>
+      <c r="M5" s="41">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="N5" s="53">
+      <c r="N5" s="52">
         <v>25</v>
       </c>
-      <c r="O5" s="28" t="e">
+      <c r="O5" s="27" t="e">
         <v>#N/A</v>
       </c>
     </row>
     <row r="6" spans="1:15">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="C6" s="20">
+      <c r="B6" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C6" s="19">
         <v>14578</v>
       </c>
-      <c r="D6" s="20">
+      <c r="D6" s="19">
         <v>5</v>
       </c>
-      <c r="E6" s="20">
-        <v>0</v>
-      </c>
-      <c r="F6" s="20">
+      <c r="E6" s="19">
+        <v>0</v>
+      </c>
+      <c r="F6" s="19">
         <v>14578</v>
       </c>
-      <c r="G6" s="50" t="s">
+      <c r="G6" s="49" t="s">
         <v>27</v>
       </c>
-      <c r="H6" s="3">
-        <v>0.1</v>
+      <c r="H6" s="2">
+        <v>0</v>
       </c>
       <c r="I6">
         <v>5648000</v>
       </c>
-      <c r="J6" s="60">
+      <c r="J6" s="59">
         <v>16725.186000000002</v>
       </c>
       <c r="K6">
         <v>2.6</v>
       </c>
-      <c r="L6" s="54">
-        <v>0</v>
-      </c>
-      <c r="M6" s="42">
+      <c r="L6" s="53">
+        <v>0</v>
+      </c>
+      <c r="M6" s="41">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="N6" s="53">
+      <c r="N6" s="52">
         <v>25</v>
       </c>
-      <c r="O6" s="28" t="e">
+      <c r="O6" s="27" t="e">
         <v>#N/A</v>
       </c>
     </row>
     <row r="7" spans="1:15">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="C7" s="20">
-        <v>0</v>
-      </c>
-      <c r="D7" s="20">
-        <v>0</v>
-      </c>
-      <c r="E7" s="20">
-        <v>0</v>
-      </c>
-      <c r="F7" s="20">
+      <c r="B7" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7" s="19">
+        <v>0</v>
+      </c>
+      <c r="D7" s="19">
+        <v>0</v>
+      </c>
+      <c r="E7" s="19">
+        <v>0</v>
+      </c>
+      <c r="F7" s="19">
         <v>100000</v>
       </c>
-      <c r="G7" s="50" t="s">
+      <c r="G7" s="49" t="s">
         <v>27</v>
       </c>
-      <c r="H7" s="51">
+      <c r="H7" s="50">
         <v>0.5</v>
       </c>
-      <c r="I7" s="53">
+      <c r="I7" s="52">
         <v>3791028.3572399998</v>
       </c>
-      <c r="J7" s="53">
+      <c r="J7" s="52">
         <v>84183.129702000006</v>
       </c>
-      <c r="K7" s="53">
+      <c r="K7" s="52">
         <v>6.75</v>
       </c>
-      <c r="L7" s="54">
-        <v>0</v>
-      </c>
-      <c r="M7" s="42">
+      <c r="L7" s="53">
+        <v>0</v>
+      </c>
+      <c r="M7" s="41">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="N7" s="53">
+      <c r="N7" s="52">
         <v>40</v>
       </c>
-      <c r="O7" s="28" t="e">
+      <c r="O7" s="27" t="e">
         <v>#N/A</v>
       </c>
     </row>
     <row r="8" spans="1:15">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B8" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="C8" s="20">
-        <v>0</v>
-      </c>
-      <c r="D8" s="20">
-        <v>0</v>
-      </c>
-      <c r="E8" s="20">
-        <v>0</v>
-      </c>
-      <c r="F8" s="20">
+      <c r="B8" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="C8" s="19">
+        <v>0</v>
+      </c>
+      <c r="D8" s="19">
+        <v>0</v>
+      </c>
+      <c r="E8" s="19">
+        <v>0</v>
+      </c>
+      <c r="F8" s="19">
         <v>100000</v>
       </c>
-      <c r="G8" s="50" t="s">
+      <c r="G8" s="49" t="s">
         <v>27</v>
       </c>
-      <c r="H8" s="51">
+      <c r="H8" s="50">
         <v>0.65</v>
       </c>
-      <c r="I8" s="53">
+      <c r="I8" s="52">
         <v>4014030.0248799999</v>
       </c>
-      <c r="J8" s="53">
+      <c r="J8" s="52">
         <v>76489.572146799997</v>
       </c>
-      <c r="K8" s="53">
+      <c r="K8" s="52">
         <v>6.96</v>
       </c>
-      <c r="L8" s="54">
-        <v>0</v>
-      </c>
-      <c r="M8" s="42">
+      <c r="L8" s="53">
+        <v>0</v>
+      </c>
+      <c r="M8" s="41">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="N8" s="53">
+      <c r="N8" s="52">
         <v>40</v>
       </c>
-      <c r="O8" s="28" t="e">
+      <c r="O8" s="27" t="e">
         <v>#N/A</v>
       </c>
     </row>
     <row r="9" spans="1:15">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="C9" s="20">
-        <v>0</v>
-      </c>
-      <c r="D9" s="20">
-        <v>0</v>
-      </c>
-      <c r="E9" s="20">
-        <v>0</v>
-      </c>
-      <c r="F9" s="20">
+      <c r="B9" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C9" s="19">
+        <v>0</v>
+      </c>
+      <c r="D9" s="19">
+        <v>0</v>
+      </c>
+      <c r="E9" s="19">
+        <v>0</v>
+      </c>
+      <c r="F9" s="19">
         <v>100000</v>
       </c>
-      <c r="G9" s="50" t="s">
+      <c r="G9" s="49" t="s">
         <v>27</v>
       </c>
-      <c r="H9" s="3">
+      <c r="H9" s="2">
         <v>0.5</v>
       </c>
-      <c r="I9" s="53">
+      <c r="I9" s="52">
         <v>1951271.6999999997</v>
       </c>
-      <c r="J9" s="53">
+      <c r="J9" s="52">
         <v>45715.5</v>
       </c>
-      <c r="K9" s="53">
+      <c r="K9" s="52">
         <v>3.46</v>
       </c>
-      <c r="L9" s="54">
-        <v>0</v>
-      </c>
-      <c r="M9" s="42">
+      <c r="L9" s="53">
+        <v>0</v>
+      </c>
+      <c r="M9" s="41">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="N9" s="53">
+      <c r="N9" s="52">
         <v>25</v>
       </c>
-      <c r="O9" s="28" t="e">
+      <c r="O9" s="27" t="e">
         <v>#N/A</v>
       </c>
     </row>
     <row r="10" spans="1:15">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B10" s="49" t="s">
+      <c r="B10" s="48" t="s">
         <v>88</v>
       </c>
-      <c r="C10" s="20">
+      <c r="C10" s="19">
         <v>94198</v>
       </c>
-      <c r="D10" s="20">
+      <c r="D10" s="19">
         <v>55</v>
       </c>
-      <c r="E10" s="20">
-        <v>0</v>
-      </c>
-      <c r="F10" s="20">
+      <c r="E10" s="19">
+        <v>0</v>
+      </c>
+      <c r="F10" s="19">
         <v>94198</v>
       </c>
-      <c r="G10" s="50" t="s">
+      <c r="G10" s="49" t="s">
         <v>27</v>
       </c>
-      <c r="H10" s="3">
+      <c r="H10" s="2">
         <v>0.8</v>
       </c>
-      <c r="I10" s="52">
+      <c r="I10" s="51">
         <v>5909565.7200000007</v>
       </c>
-      <c r="J10" s="55">
+      <c r="J10" s="54">
         <v>133801.48800000001</v>
       </c>
-      <c r="K10" s="52">
+      <c r="K10" s="51">
         <v>7.1</v>
       </c>
-      <c r="L10" s="53">
-        <v>0</v>
-      </c>
-      <c r="M10" s="42">
+      <c r="L10" s="52">
+        <v>0</v>
+      </c>
+      <c r="M10" s="41">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="N10" s="53">
+      <c r="N10" s="52">
         <v>60</v>
       </c>
-      <c r="O10" s="28" t="e">
+      <c r="O10" s="27" t="e">
         <v>#N/A</v>
       </c>
     </row>
     <row r="11" spans="1:15">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B11" s="49" t="s">
+      <c r="B11" s="48" t="s">
         <v>84</v>
       </c>
-      <c r="C11" s="20">
+      <c r="C11" s="19">
         <v>46703</v>
       </c>
-      <c r="D11" s="20">
+      <c r="D11" s="19">
         <v>30</v>
       </c>
-      <c r="E11" s="20">
-        <v>0</v>
-      </c>
-      <c r="F11" s="20">
+      <c r="E11" s="19">
+        <v>0</v>
+      </c>
+      <c r="F11" s="19">
         <v>46703</v>
       </c>
-      <c r="G11" s="50" t="s">
+      <c r="G11" s="49" t="s">
         <v>27</v>
       </c>
-      <c r="H11" s="3">
+      <c r="H11" s="2">
         <v>0.3</v>
       </c>
-      <c r="I11" s="52">
+      <c r="I11" s="51">
         <v>2731780.3800000004</v>
       </c>
-      <c r="J11" s="52">
+      <c r="J11" s="51">
         <v>9923.6103600000006</v>
       </c>
-      <c r="K11" s="52">
-        <v>0</v>
-      </c>
-      <c r="L11" s="53">
-        <v>0</v>
-      </c>
-      <c r="M11" s="42">
+      <c r="K11" s="51">
+        <v>0</v>
+      </c>
+      <c r="L11" s="52">
+        <v>0</v>
+      </c>
+      <c r="M11" s="41">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="N11" s="53">
+      <c r="N11" s="52">
         <v>60</v>
       </c>
-      <c r="O11" s="28" t="e">
+      <c r="O11" s="27" t="e">
         <v>#N/A</v>
       </c>
     </row>
     <row r="12" spans="1:15">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B12" s="49" t="s">
+      <c r="B12" s="48" t="s">
         <v>85</v>
       </c>
-      <c r="C12" s="20">
+      <c r="C12" s="19">
         <v>61218</v>
       </c>
-      <c r="D12" s="20">
+      <c r="D12" s="19">
         <v>30</v>
       </c>
-      <c r="E12" s="20">
-        <v>0</v>
-      </c>
-      <c r="F12" s="20">
+      <c r="E12" s="19">
+        <v>0</v>
+      </c>
+      <c r="F12" s="19">
         <v>61218</v>
       </c>
-      <c r="G12" s="50" t="s">
+      <c r="G12" s="49" t="s">
         <v>27</v>
       </c>
-      <c r="H12" s="3">
+      <c r="H12" s="2">
         <v>0.3</v>
       </c>
-      <c r="I12" s="53">
+      <c r="I12" s="52">
         <v>3345037.2</v>
       </c>
-      <c r="J12" s="53">
+      <c r="J12" s="52">
         <v>28432.799999999999</v>
       </c>
-      <c r="K12" s="53">
+      <c r="K12" s="52">
         <v>0.35699999999999998</v>
       </c>
-      <c r="L12" s="53">
-        <v>0</v>
-      </c>
-      <c r="M12" s="42">
+      <c r="L12" s="52">
+        <v>0</v>
+      </c>
+      <c r="M12" s="41">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="N12" s="53">
+      <c r="N12" s="52">
         <v>50</v>
       </c>
-      <c r="O12" s="28" t="e">
+      <c r="O12" s="27" t="e">
         <v>#N/A</v>
       </c>
     </row>
     <row r="13" spans="1:15">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B13" s="49" t="s">
+      <c r="B13" s="48" t="s">
         <v>89</v>
       </c>
-      <c r="C13" s="20">
+      <c r="C13" s="19">
         <v>18651</v>
       </c>
-      <c r="D13" s="20">
+      <c r="D13" s="19">
         <v>10</v>
       </c>
-      <c r="E13" s="20">
-        <v>0</v>
-      </c>
-      <c r="F13" s="20">
+      <c r="E13" s="19">
+        <v>0</v>
+      </c>
+      <c r="F13" s="19">
         <v>999999</v>
       </c>
-      <c r="G13" s="50" t="s">
+      <c r="G13" s="49" t="s">
         <v>27</v>
       </c>
-      <c r="H13" s="3">
-        <v>0.8</v>
-      </c>
-      <c r="I13" s="56">
+      <c r="H13" s="2">
+        <v>0.44</v>
+      </c>
+      <c r="I13" s="55">
         <v>5648000</v>
       </c>
-      <c r="J13" s="56">
-        <v>0</v>
-      </c>
-      <c r="K13" s="56">
+      <c r="J13" s="55">
+        <v>0</v>
+      </c>
+      <c r="K13" s="55">
         <v>44.2</v>
       </c>
-      <c r="L13" s="53">
-        <v>0</v>
-      </c>
-      <c r="M13" s="42">
+      <c r="L13" s="52">
+        <v>0</v>
+      </c>
+      <c r="M13" s="41">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="N13" s="53">
+      <c r="N13" s="52">
         <v>25</v>
       </c>
-      <c r="O13" s="28" t="e">
+      <c r="O13" s="27" t="e">
         <v>#N/A</v>
       </c>
     </row>
@@ -4157,12 +4211,12 @@
   <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="16.33203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.44140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.6640625" style="21" customWidth="1"/>
-    <col min="5" max="5" width="18.5546875" style="21" customWidth="1"/>
-    <col min="6" max="16384" width="11.44140625" style="3"/>
+    <col min="1" max="1" width="16.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.6640625" style="20" customWidth="1"/>
+    <col min="5" max="5" width="18.5546875" style="20" customWidth="1"/>
+    <col min="6" max="16384" width="11.44140625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" customFormat="1">
@@ -4175,571 +4229,571 @@
       <c r="C1" t="s">
         <v>37</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="D1" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="E1" s="18" t="s">
+      <c r="E1" s="17" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D2" s="23">
+        <v>2.4390243902439024</v>
+      </c>
+      <c r="E2" s="23">
+        <v>2.4390243902439024</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D3" s="23">
+        <v>1</v>
+      </c>
+      <c r="E3" s="23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D4" s="23">
+        <v>0.88536585365853659</v>
+      </c>
+      <c r="E4" s="23">
+        <v>0.88536585365853659</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="56" t="s">
+        <v>87</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D5" s="23">
+        <v>2.04</v>
+      </c>
+      <c r="E5" s="23">
+        <v>2.04</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" s="56" t="s">
+        <v>87</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D6" s="23">
+        <v>1</v>
+      </c>
+      <c r="E6" s="23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="56" t="s">
+        <v>87</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D7" s="23">
+        <v>0.41208</v>
+      </c>
+      <c r="E7" s="23">
+        <v>0.41208</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" s="56" t="s">
+        <v>89</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D8" s="23">
+        <v>2.8571428571428572</v>
+      </c>
+      <c r="E8" s="23">
+        <v>2.8571428571428572</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" s="56" t="s">
+        <v>89</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D9" s="23">
+        <v>1</v>
+      </c>
+      <c r="E9" s="23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="56" t="s">
+        <v>89</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D10" s="23">
+        <v>0</v>
+      </c>
+      <c r="E10" s="23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" s="56" t="s">
+        <v>88</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D11" s="23">
+        <v>2.6315789473684212</v>
+      </c>
+      <c r="E11" s="23">
+        <v>2.6315789473684212</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" s="56" t="s">
+        <v>88</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D12" s="23">
+        <v>1</v>
+      </c>
+      <c r="E12" s="23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" s="56" t="s">
+        <v>86</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13" s="23">
+        <v>2.2222222222222223</v>
+      </c>
+      <c r="E13" s="23">
+        <v>2.2222222222222223</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" s="56" t="s">
+        <v>86</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D14" s="23">
+        <v>1</v>
+      </c>
+      <c r="E14" s="23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" s="56" t="s">
+        <v>86</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D15" s="23">
+        <v>0.75955555555555554</v>
+      </c>
+      <c r="E15" s="23">
+        <v>0.75955555555555554</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" s="56" t="s">
+        <v>84</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D16" s="23">
+        <v>1</v>
+      </c>
+      <c r="E16" s="23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" s="56" t="s">
+        <v>84</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D17" s="23">
+        <v>1</v>
+      </c>
+      <c r="E17" s="23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" s="56" t="s">
+        <v>85</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D18" s="23">
+        <v>1</v>
+      </c>
+      <c r="E18" s="23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" s="56" t="s">
+        <v>85</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D19" s="23">
+        <v>1</v>
+      </c>
+      <c r="E19" s="23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D20" s="23">
+        <v>2.7777777777777777</v>
+      </c>
+      <c r="E20" s="23">
+        <v>2.7777777777777777</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21" s="23">
+        <v>1</v>
+      </c>
+      <c r="E21" s="23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D22" s="23">
+        <v>9.4944444444444442E-2</v>
+      </c>
+      <c r="E22" s="23">
+        <v>9.4944444444444442E-2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D23" s="23">
+        <v>3.125</v>
+      </c>
+      <c r="E23" s="23">
+        <v>3.125</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5">
+      <c r="A24" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D24" s="23">
+        <v>1</v>
+      </c>
+      <c r="E24" s="23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D25" s="23">
+        <v>0.1134375</v>
+      </c>
+      <c r="E25" s="23">
+        <v>0.1134375</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26" s="56" t="s">
+        <v>96</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D26" s="23">
+        <v>2.5</v>
+      </c>
+      <c r="E26" s="23">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
+      <c r="A27" s="56" t="s">
+        <v>96</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D27" s="23">
+        <v>1</v>
+      </c>
+      <c r="E27" s="23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5">
+      <c r="A28" s="56" t="s">
+        <v>96</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D28" s="23">
+        <v>5.1250000000000004E-2</v>
+      </c>
+      <c r="E28" s="23">
+        <v>5.1250000000000004E-2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5">
+      <c r="A29" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D29" s="23">
+        <v>2.5</v>
+      </c>
+      <c r="E29" s="23">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5">
+      <c r="A30" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30" s="23">
+        <v>1</v>
+      </c>
+      <c r="E30" s="23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5">
+      <c r="A31" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D31" s="23">
+        <v>0.66749999999999998</v>
+      </c>
+      <c r="E31" s="23">
+        <v>0.66749999999999998</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5">
+      <c r="A32" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="C2" s="4" t="s">
+      <c r="B32" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C32" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D2" s="24">
-        <v>2.4390243902439024</v>
-      </c>
-      <c r="E2" s="24">
-        <v>2.4390243902439024</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" s="3" t="s">
+      <c r="D32" s="23">
+        <v>2.5</v>
+      </c>
+      <c r="E32" s="23">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5">
+      <c r="A33" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B33" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C33" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="D3" s="24">
+      <c r="D33" s="23">
         <v>1</v>
       </c>
-      <c r="E3" s="24">
+      <c r="E33" s="23">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
-      <c r="A4" s="3" t="s">
+    <row r="34" spans="1:5">
+      <c r="A34" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B34" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C34" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="D4" s="24">
-        <v>0.88536585365853659</v>
-      </c>
-      <c r="E4" s="24">
-        <v>0.88536585365853659</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5" s="57" t="s">
-        <v>87</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D5" s="24">
-        <v>2.04</v>
-      </c>
-      <c r="E5" s="24">
-        <v>2.04</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
-      <c r="A6" s="57" t="s">
-        <v>87</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D6" s="24">
-        <v>1</v>
-      </c>
-      <c r="E6" s="24">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5">
-      <c r="A7" s="57" t="s">
-        <v>87</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D7" s="24">
-        <v>0.41208</v>
-      </c>
-      <c r="E7" s="24">
-        <v>0.41208</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5">
-      <c r="A8" s="57" t="s">
-        <v>89</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D8" s="24">
-        <v>2.8571428571428572</v>
-      </c>
-      <c r="E8" s="24">
-        <v>2.8571428571428572</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5">
-      <c r="A9" s="57" t="s">
-        <v>89</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D9" s="24">
-        <v>1</v>
-      </c>
-      <c r="E9" s="24">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5">
-      <c r="A10" s="57" t="s">
-        <v>89</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D10" s="24">
-        <v>0</v>
-      </c>
-      <c r="E10" s="24">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5">
-      <c r="A11" s="57" t="s">
-        <v>88</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D11" s="24">
-        <v>2.6315789473684212</v>
-      </c>
-      <c r="E11" s="24">
-        <v>2.6315789473684212</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5">
-      <c r="A12" s="57" t="s">
-        <v>88</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D12" s="24">
-        <v>1</v>
-      </c>
-      <c r="E12" s="24">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5">
-      <c r="A13" s="57" t="s">
-        <v>86</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D13" s="24">
-        <v>2.2222222222222223</v>
-      </c>
-      <c r="E13" s="24">
-        <v>2.2222222222222223</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5">
-      <c r="A14" s="57" t="s">
-        <v>86</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D14" s="24">
-        <v>1</v>
-      </c>
-      <c r="E14" s="24">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5">
-      <c r="A15" s="57" t="s">
-        <v>86</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D15" s="24">
-        <v>0.75955555555555554</v>
-      </c>
-      <c r="E15" s="24">
-        <v>0.75955555555555554</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5">
-      <c r="A16" s="57" t="s">
-        <v>84</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D16" s="24">
-        <v>1</v>
-      </c>
-      <c r="E16" s="24">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5">
-      <c r="A17" s="57" t="s">
-        <v>84</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D17" s="24">
-        <v>1</v>
-      </c>
-      <c r="E17" s="24">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5">
-      <c r="A18" s="57" t="s">
-        <v>85</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D18" s="24">
-        <v>1</v>
-      </c>
-      <c r="E18" s="24">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5">
-      <c r="A19" s="57" t="s">
-        <v>85</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D19" s="24">
-        <v>1</v>
-      </c>
-      <c r="E19" s="24">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5">
-      <c r="A20" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D20" s="24">
-        <v>2.7777777777777777</v>
-      </c>
-      <c r="E20" s="24">
-        <v>2.7777777777777777</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5">
-      <c r="A21" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D21" s="24">
-        <v>1</v>
-      </c>
-      <c r="E21" s="24">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5">
-      <c r="A22" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D22" s="24">
-        <v>9.4944444444444442E-2</v>
-      </c>
-      <c r="E22" s="24">
-        <v>9.4944444444444442E-2</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5">
-      <c r="A23" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D23" s="24">
-        <v>3.125</v>
-      </c>
-      <c r="E23" s="24">
-        <v>3.125</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5">
-      <c r="A24" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D24" s="24">
-        <v>1</v>
-      </c>
-      <c r="E24" s="24">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5">
-      <c r="A25" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D25" s="24">
-        <v>0.1134375</v>
-      </c>
-      <c r="E25" s="24">
-        <v>0.1134375</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5">
-      <c r="A26" s="57" t="s">
-        <v>98</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D26" s="24">
-        <v>2.5</v>
-      </c>
-      <c r="E26" s="24">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5">
-      <c r="A27" s="57" t="s">
-        <v>98</v>
-      </c>
-      <c r="B27" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D27" s="24">
-        <v>1</v>
-      </c>
-      <c r="E27" s="24">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5">
-      <c r="A28" s="57" t="s">
-        <v>98</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D28" s="24">
-        <v>5.1250000000000004E-2</v>
-      </c>
-      <c r="E28" s="24">
-        <v>5.1250000000000004E-2</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5">
-      <c r="A29" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="B29" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D29" s="24">
-        <v>2.5</v>
-      </c>
-      <c r="E29" s="24">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5">
-      <c r="A30" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="B30" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D30" s="24">
-        <v>1</v>
-      </c>
-      <c r="E30" s="24">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5">
-      <c r="A31" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="B31" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D31" s="24">
+      <c r="D34" s="23">
         <v>0.66749999999999998</v>
       </c>
-      <c r="E31" s="24">
-        <v>0.66749999999999998</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5">
-      <c r="A32" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D32" s="24">
-        <v>2.5</v>
-      </c>
-      <c r="E32" s="24">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5">
-      <c r="A33" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C33" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D33" s="24">
-        <v>1</v>
-      </c>
-      <c r="E33" s="24">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5">
-      <c r="A34" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="B34" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D34" s="24">
-        <v>0.66749999999999998</v>
-      </c>
-      <c r="E34" s="24">
+      <c r="E34" s="23">
         <v>0.66749999999999998</v>
       </c>
     </row>
@@ -4966,6 +5020,20 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="E7">
+    <cfRule type="dataBar" priority="1">
+      <dataBar>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="2"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{F74817C3-D28A-45F6-A051-86E1B85965F4}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="E20:E34">
     <cfRule type="dataBar" priority="2">
       <dataBar>
@@ -4995,20 +5063,6 @@
   <conditionalFormatting sqref="F6:XFD34">
     <cfRule type="expression" dxfId="3" priority="7">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E7">
-    <cfRule type="dataBar" priority="1">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="2"/>
-        <color rgb="FF638EC6"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F74817C3-D28A-45F6-A051-86E1B85965F4}</x14:id>
-        </ext>
-      </extLst>
     </cfRule>
   </conditionalFormatting>
   <dataValidations xWindow="701" yWindow="283" count="2">
@@ -5198,6 +5252,21 @@
           <xm:sqref>E6:E7</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{F74817C3-D28A-45F6-A051-86E1B85965F4}">
+            <x14:dataBar minLength="0" maxLength="100" gradient="0">
+              <x14:cfvo type="num">
+                <xm:f>0</xm:f>
+              </x14:cfvo>
+              <x14:cfvo type="num">
+                <xm:f>2</xm:f>
+              </x14:cfvo>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>E7</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{7DACECD8-CF17-4DAC-86F1-80FDC5E5A1ED}">
             <x14:dataBar minLength="0" maxLength="100" gradient="0">
               <x14:cfvo type="num">
@@ -5224,21 +5293,6 @@
           </x14:cfRule>
           <xm:sqref>E20:E34</xm:sqref>
         </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F74817C3-D28A-45F6-A051-86E1B85965F4}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>2</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>E7</xm:sqref>
-        </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
   </extLst>
@@ -5256,12 +5310,12 @@
     <col min="1" max="2" width="10.6640625" customWidth="1"/>
     <col min="3" max="3" width="14.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="10.6640625" style="21" customWidth="1"/>
-    <col min="7" max="7" width="11.6640625" style="20" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.6640625" style="20" customWidth="1"/>
-    <col min="9" max="9" width="10.6640625" style="23" customWidth="1"/>
-    <col min="10" max="13" width="10.6640625" style="20" customWidth="1"/>
-    <col min="14" max="14" width="14.88671875" style="23" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="10.6640625" style="20" customWidth="1"/>
+    <col min="7" max="7" width="11.6640625" style="19" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.6640625" style="19" customWidth="1"/>
+    <col min="9" max="9" width="10.6640625" style="22" customWidth="1"/>
+    <col min="10" max="13" width="10.6640625" style="19" customWidth="1"/>
+    <col min="14" max="14" width="14.88671875" style="22" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="12.109375" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="10.88671875" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="15.44140625" bestFit="1" customWidth="1"/>
@@ -5280,43 +5334,43 @@
       <c r="D1" t="s">
         <v>38</v>
       </c>
-      <c r="E1" s="18" t="s">
+      <c r="E1" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="F1" s="18" t="s">
+      <c r="F1" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="G1" s="17" t="s">
+      <c r="G1" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="H1" s="17" t="s">
+      <c r="H1" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="I1" s="16" t="s">
+      <c r="I1" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="J1" s="17" t="s">
+      <c r="J1" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="17" t="s">
+      <c r="K1" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="17" t="s">
+      <c r="L1" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="16" t="s">
+      <c r="M1" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="N1" s="16" t="s">
+      <c r="N1" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="O1" s="16" t="s">
+      <c r="O1" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="P1" s="16" t="s">
+      <c r="P1" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="Q1" s="16" t="s">
+      <c r="Q1" s="15" t="s">
         <v>78</v>
       </c>
     </row>
@@ -5354,306 +5408,306 @@
   <dimension ref="A1:W4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="10.6640625" style="3" customWidth="1"/>
-    <col min="2" max="2" width="13.109375" style="3" customWidth="1"/>
-    <col min="3" max="3" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.109375" style="20" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.5546875" style="20" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.109375" style="20" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.44140625" style="20" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.88671875" style="20" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.44140625" style="20" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="10.6640625" style="23" customWidth="1"/>
-    <col min="12" max="12" width="12.44140625" style="20" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.109375" style="23" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12" style="20" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.6640625" style="23" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.44140625" style="23" bestFit="1" customWidth="1"/>
-    <col min="17" max="19" width="12.109375" style="23" customWidth="1"/>
-    <col min="20" max="20" width="14.88671875" style="23" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.6640625" style="23" customWidth="1"/>
-    <col min="22" max="22" width="12.109375" style="23" bestFit="1" customWidth="1"/>
-    <col min="23" max="16384" width="11.44140625" style="3"/>
+    <col min="1" max="1" width="10.6640625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="13.109375" style="2" customWidth="1"/>
+    <col min="3" max="3" width="13.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.109375" style="19" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.5546875" style="19" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.109375" style="19" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.44140625" style="19" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.88671875" style="19" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.44140625" style="19" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="10.6640625" style="22" customWidth="1"/>
+    <col min="12" max="12" width="12.44140625" style="19" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.109375" style="22" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12" style="19" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.6640625" style="22" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.44140625" style="22" bestFit="1" customWidth="1"/>
+    <col min="17" max="19" width="12.109375" style="22" customWidth="1"/>
+    <col min="20" max="20" width="14.88671875" style="22" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.6640625" style="22" customWidth="1"/>
+    <col min="22" max="22" width="12.109375" style="22" bestFit="1" customWidth="1"/>
+    <col min="23" max="16384" width="11.44140625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="E1" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="F1" s="17" t="s">
+      <c r="F1" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="17" t="s">
+      <c r="G1" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="H1" s="17" t="s">
+      <c r="H1" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="I1" s="17" t="s">
+      <c r="I1" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="J1" s="16" t="s">
+      <c r="J1" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="K1" s="16" t="s">
+      <c r="K1" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="L1" s="17" t="s">
+      <c r="L1" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="M1" s="16" t="s">
+      <c r="M1" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="17" t="s">
+      <c r="N1" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="O1" s="16" t="s">
+      <c r="O1" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="P1" s="16" t="s">
+      <c r="P1" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="Q1" s="16" t="s">
+      <c r="Q1" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="R1" s="16" t="s">
+      <c r="R1" s="15" t="s">
         <v>73</v>
       </c>
-      <c r="S1" s="16" t="s">
+      <c r="S1" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="T1" s="16" t="s">
+      <c r="T1" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="U1" s="16" t="s">
+      <c r="U1" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="V1" s="16" t="s">
+      <c r="V1" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="W1" s="36" t="s">
+      <c r="W1" s="35" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:23">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B2" s="41" t="s">
+      <c r="B2" s="40" t="s">
         <v>81</v>
       </c>
-      <c r="C2" s="41" t="s">
+      <c r="C2" s="40" t="s">
         <v>35</v>
       </c>
-      <c r="D2" s="39">
-        <v>0</v>
-      </c>
-      <c r="E2" s="39">
-        <v>0</v>
-      </c>
-      <c r="F2" s="39" t="s">
+      <c r="D2" s="38">
+        <v>0</v>
+      </c>
+      <c r="E2" s="38">
+        <v>0</v>
+      </c>
+      <c r="F2" s="38" t="s">
         <v>27</v>
       </c>
-      <c r="G2" s="39">
-        <v>0</v>
-      </c>
-      <c r="H2" s="39">
-        <v>0</v>
-      </c>
-      <c r="I2" s="39" t="s">
+      <c r="G2" s="38">
+        <v>0</v>
+      </c>
+      <c r="H2" s="38">
+        <v>0</v>
+      </c>
+      <c r="I2" s="38" t="s">
         <v>27</v>
       </c>
-      <c r="J2" s="44">
+      <c r="J2" s="43">
         <v>0.66</v>
       </c>
-      <c r="K2" s="43">
+      <c r="K2" s="42">
         <v>0.3</v>
       </c>
-      <c r="L2" s="44">
+      <c r="L2" s="43">
         <v>565000</v>
       </c>
-      <c r="M2" s="25">
-        <v>0</v>
-      </c>
-      <c r="N2" s="44">
+      <c r="M2" s="24">
+        <v>0</v>
+      </c>
+      <c r="N2" s="43">
         <v>12000</v>
       </c>
-      <c r="O2" s="25">
-        <v>0</v>
-      </c>
-      <c r="P2" s="25">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="25">
-        <v>0</v>
-      </c>
-      <c r="R2" s="25">
-        <v>0</v>
-      </c>
-      <c r="S2" s="42">
+      <c r="O2" s="24">
+        <v>0</v>
+      </c>
+      <c r="P2" s="24">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="24">
+        <v>0</v>
+      </c>
+      <c r="R2" s="24">
+        <v>0</v>
+      </c>
+      <c r="S2" s="41">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="T2" s="44">
+      <c r="T2" s="43">
         <v>25</v>
       </c>
-      <c r="U2" s="25">
+      <c r="U2" s="24">
         <v>0.5</v>
       </c>
-      <c r="V2" s="40">
+      <c r="V2" s="39">
         <v>3.4999999999999999E-6</v>
       </c>
-      <c r="W2" s="25"/>
+      <c r="W2" s="24"/>
     </row>
     <row r="3" spans="1:23">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B3" s="41" t="s">
+      <c r="B3" s="40" t="s">
         <v>82</v>
       </c>
-      <c r="C3" s="41" t="s">
+      <c r="C3" s="40" t="s">
         <v>35</v>
       </c>
-      <c r="D3" s="39">
-        <v>0</v>
-      </c>
-      <c r="E3" s="39">
-        <v>0</v>
-      </c>
-      <c r="F3" s="39" t="s">
+      <c r="D3" s="38">
+        <v>0</v>
+      </c>
+      <c r="E3" s="38">
+        <v>0</v>
+      </c>
+      <c r="F3" s="38" t="s">
         <v>27</v>
       </c>
-      <c r="G3" s="39">
-        <v>0</v>
-      </c>
-      <c r="H3" s="39">
-        <v>0</v>
-      </c>
-      <c r="I3" s="39" t="s">
+      <c r="G3" s="38">
+        <v>0</v>
+      </c>
+      <c r="H3" s="38">
+        <v>0</v>
+      </c>
+      <c r="I3" s="38" t="s">
         <v>27</v>
       </c>
-      <c r="J3" s="45">
+      <c r="J3" s="44">
         <v>0.9</v>
       </c>
-      <c r="K3" s="45">
+      <c r="K3" s="44">
         <v>0.9</v>
       </c>
-      <c r="L3" s="44">
+      <c r="L3" s="43">
         <v>4412341</v>
       </c>
-      <c r="M3" s="44">
-        <v>0</v>
-      </c>
-      <c r="N3" s="44">
+      <c r="M3" s="43">
+        <v>0</v>
+      </c>
+      <c r="N3" s="43">
         <v>34383</v>
       </c>
-      <c r="O3" s="44">
+      <c r="O3" s="43">
         <f>0.05*M3</f>
         <v>0</v>
       </c>
-      <c r="P3" s="44">
+      <c r="P3" s="43">
         <v>8.1999999999999993</v>
       </c>
-      <c r="Q3" s="25">
-        <v>0</v>
-      </c>
-      <c r="R3" s="25">
-        <v>0</v>
-      </c>
-      <c r="S3" s="42">
+      <c r="Q3" s="24">
+        <v>0</v>
+      </c>
+      <c r="R3" s="24">
+        <v>0</v>
+      </c>
+      <c r="S3" s="41">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="T3" s="44">
+      <c r="T3" s="43">
         <v>25</v>
       </c>
-      <c r="U3" s="25">
+      <c r="U3" s="24">
         <v>0.5</v>
       </c>
-      <c r="V3" s="46">
-        <v>0</v>
-      </c>
-      <c r="W3" s="25"/>
+      <c r="V3" s="45">
+        <v>0</v>
+      </c>
+      <c r="W3" s="24"/>
     </row>
     <row r="4" spans="1:23">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B4" s="47" t="s">
+      <c r="B4" s="46" t="s">
         <v>83</v>
       </c>
-      <c r="C4" s="41" t="s">
+      <c r="C4" s="40" t="s">
         <v>35</v>
       </c>
-      <c r="D4" s="39">
-        <v>0</v>
-      </c>
-      <c r="E4" s="39">
-        <v>0</v>
-      </c>
-      <c r="F4" s="39" t="s">
+      <c r="D4" s="38">
+        <v>0</v>
+      </c>
+      <c r="E4" s="38">
+        <v>0</v>
+      </c>
+      <c r="F4" s="38" t="s">
         <v>27</v>
       </c>
-      <c r="G4" s="39">
-        <v>0</v>
-      </c>
-      <c r="H4" s="39">
-        <v>0</v>
-      </c>
-      <c r="I4" s="39" t="s">
+      <c r="G4" s="38">
+        <v>0</v>
+      </c>
+      <c r="H4" s="38">
+        <v>0</v>
+      </c>
+      <c r="I4" s="38" t="s">
         <v>27</v>
       </c>
-      <c r="J4" s="48">
+      <c r="J4" s="47">
         <v>0.86</v>
       </c>
-      <c r="K4" s="48">
+      <c r="K4" s="47">
         <v>0.86</v>
       </c>
-      <c r="L4" s="44">
-        <v>0</v>
-      </c>
-      <c r="M4" s="44">
+      <c r="L4" s="43">
+        <v>0</v>
+      </c>
+      <c r="M4" s="43">
         <v>520000</v>
       </c>
-      <c r="N4" s="44">
-        <v>0</v>
-      </c>
-      <c r="O4" s="44">
+      <c r="N4" s="43">
+        <v>0</v>
+      </c>
+      <c r="O4" s="43">
         <v>5000</v>
       </c>
-      <c r="P4" s="44">
+      <c r="P4" s="43">
         <v>0.4</v>
       </c>
-      <c r="Q4" s="25">
-        <v>0</v>
-      </c>
-      <c r="R4" s="25">
-        <v>0</v>
-      </c>
-      <c r="S4" s="42">
+      <c r="Q4" s="24">
+        <v>0</v>
+      </c>
+      <c r="R4" s="24">
+        <v>0</v>
+      </c>
+      <c r="S4" s="41">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="T4" s="48">
+      <c r="T4" s="47">
         <v>15</v>
       </c>
-      <c r="U4" s="25">
+      <c r="U4" s="24">
         <v>0.5</v>
       </c>
-      <c r="V4" s="25">
-        <v>0</v>
-      </c>
-      <c r="W4" s="25"/>
+      <c r="V4" s="24">
+        <v>0</v>
+      </c>
+      <c r="W4" s="24"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:U1" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
@@ -5706,31 +5760,31 @@
     <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.33203125" style="35" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.33203125" style="34" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.44140625" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="C1" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="D1" s="34" t="s">
+      <c r="D1" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="E1" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="F1" s="17" t="s">
+      <c r="F1" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="G1" s="17" t="s">
+      <c r="G1" s="16" t="s">
         <v>53</v>
       </c>
     </row>
@@ -5778,29 +5832,29 @@
   <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="11.44140625" style="2"/>
-    <col min="2" max="2" width="12.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="11.44140625" style="2"/>
+    <col min="1" max="1" width="11.44140625" style="1"/>
+    <col min="2" max="2" width="12.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="16384" width="11.44140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
-      <c r="A1" s="13" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="6" t="s">
+      <c r="A1" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="5">
-        <v>0</v>
-      </c>
-      <c r="B2" s="26">
+      <c r="A2" s="4">
+        <v>0</v>
+      </c>
+      <c r="B2" s="25">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3" s="5">
+      <c r="A3" s="4">
         <v>1</v>
       </c>
       <c r="B3">
@@ -5808,7 +5862,7 @@
       </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4" s="5">
+      <c r="A4" s="4">
         <v>2</v>
       </c>
       <c r="B4">
@@ -5816,7 +5870,7 @@
       </c>
     </row>
     <row r="5" spans="1:2">
-      <c r="A5" s="5">
+      <c r="A5" s="4">
         <v>3</v>
       </c>
       <c r="B5">
@@ -5824,7 +5878,7 @@
       </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6" s="5">
+      <c r="A6" s="4">
         <v>4</v>
       </c>
       <c r="B6">
@@ -5832,7 +5886,7 @@
       </c>
     </row>
     <row r="7" spans="1:2">
-      <c r="A7" s="5">
+      <c r="A7" s="4">
         <v>5</v>
       </c>
       <c r="B7">
@@ -5840,7 +5894,7 @@
       </c>
     </row>
     <row r="8" spans="1:2">
-      <c r="A8" s="5">
+      <c r="A8" s="4">
         <v>6</v>
       </c>
       <c r="B8">
@@ -5848,7 +5902,7 @@
       </c>
     </row>
     <row r="9" spans="1:2">
-      <c r="A9" s="5">
+      <c r="A9" s="4">
         <v>7</v>
       </c>
       <c r="B9">
@@ -5856,7 +5910,7 @@
       </c>
     </row>
     <row r="10" spans="1:2">
-      <c r="A10" s="5">
+      <c r="A10" s="4">
         <v>8</v>
       </c>
       <c r="B10">
@@ -5864,7 +5918,7 @@
       </c>
     </row>
     <row r="11" spans="1:2">
-      <c r="A11" s="5">
+      <c r="A11" s="4">
         <v>9</v>
       </c>
       <c r="B11">
@@ -5872,7 +5926,7 @@
       </c>
     </row>
     <row r="12" spans="1:2">
-      <c r="A12" s="5">
+      <c r="A12" s="4">
         <v>10</v>
       </c>
       <c r="B12">
@@ -5880,7 +5934,7 @@
       </c>
     </row>
     <row r="13" spans="1:2">
-      <c r="A13" s="5">
+      <c r="A13" s="4">
         <v>11</v>
       </c>
       <c r="B13">
@@ -5888,7 +5942,7 @@
       </c>
     </row>
     <row r="14" spans="1:2">
-      <c r="A14" s="5">
+      <c r="A14" s="4">
         <v>12</v>
       </c>
       <c r="B14">

</xml_diff>